<commit_message>
demo: cadrage « exemple d'une sortie en exclusivité » (bandeau + ligne) ; outreach: email Raidillon (prochaine sortie, place au calendrier)
</commit_message>
<xml_diff>
--- a/outreach/pipeline.xlsx
+++ b/outreach/pipeline.xlsx
@@ -359,7 +359,7 @@
     <t xml:space="preserve">/demo/raidillon-55</t>
   </si>
   <si>
-    <t xml:space="preserve">Cœur sous plancher → édition spéciale only. Belge</t>
+    <t xml:space="preserve">Démo /demo/raidillon-55 · email_raidillon.md (hello@raidillon.com). Cœur sous plancher → édition spéciale. Belge. Pitch = prochaine sortie en exclu (calendrier)</t>
   </si>
   <si>
     <t xml:space="preserve">Col&amp;MacArthur</t>
@@ -1545,7 +1545,7 @@
         <v>109</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>

</xml_diff>